<commit_message>
Add 'App ↔ Pool ↔ RBAC' sheet sourced from workloads.json
</commit_message>
<xml_diff>
--- a/docs/app-registrations.xlsx
+++ b/docs/app-registrations.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Registrations" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App ↔ Pool ↔ RBAC" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +35,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Menlo"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -80,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,6 +103,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1806,4 +1814,992 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Env</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Workload</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Entra App Registration</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Confluent Identity Pool</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Pool filter (templated)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Write topics</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Read topics</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Manage topics (DeveloperManage)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Consumer groups (DeveloperRead)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Kafka cluster</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="117" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>mergerarb</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>madam</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-dev-mergerarb-madam</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-dev-mergerarb-madam</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>exact:
+  • dev.deal.calc.mergerarb.json
+  • dev.deal.mergerarb.compact.json
+  • dev.deal.calc.mergerarb.avro
+  • dev.deal.mergerarb.compact.avro
+  • dev.deal.calc.mergerarb.v2.json
+  • dev.deal.mergerarb.compact.v2.json
+  • dev.deal.calc.mergerarb.v2.avro
+  • dev.deal.mergerarb.compact.v2.avro</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>exact:
+  • dev.deal.calc.mergerarb.json
+  • dev.deal.mergerarb.compact.json
+  • dev.deal.calc.mergerarb.avro
+  • dev.deal.mergerarb.compact.avro
+  • dev.deal.calc.mergerarb.v2.json
+  • dev.deal.mergerarb.compact.v2.json
+  • dev.deal.calc.mergerarb.v2.avro
+  • dev.deal.mergerarb.compact.v2.avro</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr"/>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • dk-confluent-dev-mergerarb-madam-</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>lkc-1o1jkv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="156" customHeight="1">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>writer</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-dev-position-writer</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-dev-position-writer</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • dev.transaction.oms.
+  • dev2.transaction.oms.
+  • dev.transactionallocation.oms.
+  • dev2.transactionallocation.oms.
+  • dev.asoftransactionallocation.oms.
+  • dev.sod.position.
+  • dev2.sod.position.
+  • dev.position.
+  • dev2.position.
+  • dev.referencedata.
+  • dev2.referencedata.</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr"/>
+      <c r="J3" s="7" t="inlineStr"/>
+      <c r="K3" s="7" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>lkc-1o1jkv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="143" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>reader</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-dev-position-reader</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-dev-position-reader</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr"/>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • dev.deal.
+  • dev2.deal.
+  • dev.security.
+  • dev2.security.
+  • dev.manager.
+  • dev2.manager.
+  • dev.fund.
+  • dev2.fund.
+  • dev.referencedata.
+  • dev2.referencedata.</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr"/>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • dk-confluent-dev-position-reader-</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>lkc-1o1jkv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="117" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>tft</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>writer</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-dev-tft-writer</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-dev-tft-writer</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • dev.deal.
+  • dev2.deal.
+  • dev.security.
+  • dev2.security.
+  • dev.manager.
+  • dev2.manager.
+  • dev.fund.
+  • dev2.fund.</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr"/>
+      <c r="J5" s="7" t="inlineStr"/>
+      <c r="K5" s="7" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>lkc-1o1jkv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="39" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ibconnect</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-dev-ibconnect-connector</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-dev-ibconnect-connector</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • dev.ibconnect.streams.avro
+  • dev.ibconnect.rawstreams.json</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr"/>
+      <c r="J6" s="7" t="inlineStr"/>
+      <c r="K6" s="7" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>lkc-1o1jkv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="117" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>uat</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>mergerarb</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>madam</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-uat-mergerarb-madam</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-uat-mergerarb-madam</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>exact:
+  • uat.deal.calc.mergerarb.json
+  • uat.deal.mergerarb.compact.json
+  • uat.deal.calc.mergerarb.avro
+  • uat.deal.mergerarb.compact.avro
+  • uat.deal.calc.mergerarb.v2.json
+  • uat.deal.mergerarb.compact.v2.json
+  • uat.deal.calc.mergerarb.v2.avro
+  • uat.deal.mergerarb.compact.v2.avro</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>exact:
+  • uat.deal.calc.mergerarb.json
+  • uat.deal.mergerarb.compact.json
+  • uat.deal.calc.mergerarb.avro
+  • uat.deal.mergerarb.compact.avro
+  • uat.deal.calc.mergerarb.v2.json
+  • uat.deal.mergerarb.compact.v2.json
+  • uat.deal.calc.mergerarb.v2.avro
+  • uat.deal.mergerarb.compact.v2.avro</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr"/>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • dk-confluent-uat-mergerarb-madam-</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>lkc-1o1jkv</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="156" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>uat</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>writer</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-uat-position-writer</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-uat-position-writer</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • uat.transaction.oms.
+  • uat2.transaction.oms.
+  • uat.transactionallocation.oms.
+  • uat2.transactionallocation.oms.
+  • uat.asoftransactionallocation.oms.
+  • uat.sod.position.
+  • uat2.sod.position.
+  • uat.position.
+  • uat2.position.
+  • uat.referencedata.
+  • uat2.referencedata.</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr"/>
+      <c r="J8" s="7" t="inlineStr"/>
+      <c r="K8" s="7" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>lkc-1o1jkv</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="156" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>uat</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>reader</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-uat-position-reader</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-uat-position-reader</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • cdc.uat.position.
+  • uat.deal.
+  • uat.security.
+  • uat.manager.
+  • uat.fund.
+  • uat2.deal.
+  • uat2.security.
+  • uat2.manager.
+  • uat2.fund.
+  • uat.referencedata.
+  • uat2.referencedata.</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr"/>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • dk-confluent-uat-position-reader-</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>lkc-1o1jkv</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="117" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>uat</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>tft</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>writer</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-uat-tft-writer</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-uat-tft-writer</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • uat.deal.
+  • uat.security.
+  • uat.manager.
+  • uat.fund.
+  • uat2.deal.
+  • uat2.security.
+  • uat2.manager.
+  • uat2.fund.</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr"/>
+      <c r="J10" s="7" t="inlineStr"/>
+      <c r="K10" s="7" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>lkc-1o1jkv</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="39" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>uat</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>ibconnect</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-uat-ibconnect-connector</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-uat-ibconnect-connector</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • uat.ibconnect.streams.avro
+  • uat.ibconnect.rawstreams.json</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr"/>
+      <c r="J11" s="7" t="inlineStr"/>
+      <c r="K11" s="7" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>lkc-1o1jkv</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>prd</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>mergerarb</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>madam</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-prd-mergerarb-madam</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-prd-mergerarb-madam</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>exact:
+  • REPLACE_WITH_PRD_MERGERARB_TOPIC_1</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>exact:
+  • REPLACE_WITH_PRD_MERGERARB_TOPIC_1</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr"/>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • dk-confluent-prd-mergerarb-madam-</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>lkc-wxdwk9</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>prd</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>writer</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-prd-position-writer</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-prd-position-writer</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • REPLACE_WITH_PRD_POSITION_WRITER_PREFIX</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr"/>
+      <c r="J13" s="7" t="inlineStr"/>
+      <c r="K13" s="7" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>lkc-wxdwk9</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>prd</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>position</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>reader</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-prd-position-reader</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-prd-position-reader</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr"/>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • REPLACE_WITH_PRD_POSITION_READER_PREFIX</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr"/>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • dk-confluent-prd-position-reader-</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>lkc-wxdwk9</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>prd</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>tft</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>writer</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-prd-tft-writer</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-prd-tft-writer</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • REPLACE_WITH_PRD_TFT_WRITER_PREFIX</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr"/>
+      <c r="J15" s="7" t="inlineStr"/>
+      <c r="K15" s="7" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>lkc-wxdwk9</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>prd</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>ibconnect</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>connector</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-prd-ibconnect-connector</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>dk-confluent-prd-ibconnect-connector</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>claims.tid == "7bab0bc1-bb61-48d7-b2d4-79825c2ac6b8" &amp;&amp; claims.aud == "&lt;Application (client) ID GUID&gt;"</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>prefix:
+  • REPLACE_WITH_PRD_IBCONNECT_PREFIX</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr"/>
+      <c r="J16" s="7" t="inlineStr"/>
+      <c r="K16" s="7" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>lkc-wxdwk9</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>prefix: CRN topic=&lt;value&gt;*  (matches all topics beginning with &lt;value&gt;)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>exact:  CRN topic=&lt;value&gt;   (matches that topic only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Pool filter's aud is the Application (client) ID GUID (v2 Entra token shape) — no api:// prefix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Source of truth: terraform/live/&lt;env&gt;/workloads.json — re-run this generator after edits.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>